<commit_message>
TCD example: confirm BBS as Bachelors, explain Faster TAT in the notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/TCD_Example_Upload.xlsx
+++ b/docs/TCD_Example_Upload.xlsx
@@ -3023,7 +3023,7 @@
         <v>degree_level</v>
       </c>
       <c r="B6" t="str">
-        <v>BBS Global Business (Bachelor in Business Studies, 48 months) was labelled Masters in the source; set to 0 (Bachelors). CONFIRM</v>
+        <v>BBS Global Business (Bachelor in Business Studies, 48 months) was labelled Masters in the source; set to 0 (Bachelors), confirmed</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -3155,7 +3155,7 @@
         <v>has_faster_tat</v>
       </c>
       <c r="B18" t="str">
-        <v>Source said "4 to 8 weeks", which isn't Yes/No. Set to No. CONFIRM whether TCD counts as faster turnaround</v>
+        <v>Source said "4 to 8 weeks" (TCD's normal decision time). Set to No: Faster TAT means the university decides applications faster than usual, and shows as a "Faster TAT" badge in Uni Assist</v>
       </c>
       <c r="C18">
         <v>25</v>

</xml_diff>